<commit_message>
Updated Booked Hours and included Important Topics discussed and brought up in group meeting
</commit_message>
<xml_diff>
--- a/Documentation/Week 7/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 7/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 7/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9CFA659-C372-4529-98E1-69B431E89C4E}"/>
+  <xr:revisionPtr revIDLastSave="254" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F3EF72F-3C3C-4D81-A67F-2F8FF8779BD2}"/>
   <bookViews>
     <workbookView xWindow="16980" yWindow="780" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="30">
   <si>
     <t>Wk</t>
   </si>
@@ -490,6 +490,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1952,21 +1956,35 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="4"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="5"/>
-      <c r="G38" s="6" t="str">
+      <c r="A38" s="1">
+        <v>7</v>
+      </c>
+      <c r="B38" s="4">
+        <v>44812</v>
+      </c>
+      <c r="C38" s="5">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D38" s="4">
+        <v>44812</v>
+      </c>
+      <c r="E38" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G38" s="6">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H38" s="1" t="str">
+        <v>0.99999999994179234</v>
+      </c>
+      <c r="H38" s="1">
         <f t="shared" si="4"/>
-        <v xml:space="preserve"> </v>
+        <v>30.749999999825377</v>
       </c>
       <c r="I38" s="1">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.99999999994179234</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>